<commit_message>
Complete EXP-013 top-20 adjudication
</commit_message>
<xml_diff>
--- a/Patent_AI_Experiment_Dashboard_Canonical.xlsx
+++ b/Patent_AI_Experiment_Dashboard_Canonical.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rcd8ca2a8a7204daa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" r:id="R3311dc9c792040f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Inputs" sheetId="3" r:id="Rc5a5c7597a294ff5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Versions" sheetId="4" r:id="R1a933fbaceed4c8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Definitions" sheetId="5" r:id="R8611dd6affaa40c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R518a98c7c2e74836"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" r:id="Rbd23c3c2892147f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Inputs" sheetId="3" r:id="R1147256ed16e40e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Versions" sheetId="4" r:id="Rce7c9615e51c4fd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Definitions" sheetId="5" r:id="R460990d3bb2646d0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,12 +17,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="0%"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="202" formatCode="$0.00"/>
     <x:numFmt numFmtId="203" formatCode="0.0"/>
     <x:numFmt numFmtId="204" formatCode="0"/>
+    <x:numFmt numFmtId="205" formatCode="0.0%"/>
+    <x:numFmt numFmtId="206" formatCode="General"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -47,7 +49,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +81,11 @@
         <x:fgColor rgb="FF4472C4"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -87,7 +94,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="46">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -176,6 +183,34 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -594,7 +629,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Last Validated Experiment</x:v>
+        <x:v>Current Experiment</x:v>
       </x:c>
       <x:c r="B8" t="str">
         <x:v>EXP-013</x:v>
@@ -618,8 +653,8 @@
         <x:v>Best Precision@20</x:v>
       </x:c>
       <x:c r="E9" s="18" t="n">
-        <x:f>MAX('Experiment Log'!N2:N200)</x:f>
-        <x:v>0</x:v>
+        <x:f>IF(COUNT('Experiment Log'!N2:N200)=0,"N/A",MAX('Experiment Log'!N2:N200))</x:f>
+        <x:v>0.45</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -757,30 +792,30 @@
         <x:v>BASELINE</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" t="str">
+    <x:row r="22" ht="70" customHeight="1">
+      <x:c r="A22" s="24" t="str">
         <x:v>EXP-013</x:v>
       </x:c>
-      <x:c r="B22" t="str">
+      <x:c r="B22" s="24" t="str">
         <x:v>Blind title/abstract reranking</x:v>
       </x:c>
-      <x:c r="C22" t="str">
-        <x:v>Recall@100 4/10; median GOLD rank 90.5</x:v>
-      </x:c>
-      <x:c r="D22" t="str">
+      <x:c r="C22" s="24" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D22" s="24" t="str">
         <x:v>20%</x:v>
       </x:c>
-      <x:c r="E22" t="str">
+      <x:c r="E22" s="24" t="str">
         <x:v>40%</x:v>
       </x:c>
-      <x:c r="F22" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="G22" t="str">
+      <x:c r="F22" s="31" t="n">
+        <x:v>0.45</x:v>
+      </x:c>
+      <x:c r="G22" s="24" t="str">
         <x:v>90.5</x:v>
       </x:c>
-      <x:c r="H22" t="str">
-        <x:v>INCONCLUSIVE</x:v>
+      <x:c r="H22" s="24" t="str">
+        <x:v>HOLD / INCONCLUSIVE</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -801,12 +836,373 @@
         <x:v>PARTIALLY_VALIDATED</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" ht="40" customHeight="1">
+      <x:c r="A25" s="49" t="str">
+        <x:v>EXP-013 completed adjudication</x:v>
+      </x:c>
+      <x:c r="B25" s="49" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C25" s="49" t="str">
+        <x:v>Scope / limitation</x:v>
+      </x:c>
+      <x:c r="D25" s="49"/>
+      <x:c r="E25" s="49"/>
+      <x:c r="F25" s="49"/>
+      <x:c r="G25" s="49"/>
+      <x:c r="H25" s="49"/>
+    </x:row>
+    <x:row r="26" ht="42" customHeight="1">
+      <x:c r="A26" s="52" t="str">
+        <x:v>Newly adjudicated publications</x:v>
+      </x:c>
+      <x:c r="B26" s="55" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C26" s="52" t="str">
+        <x:v>Completed analyst decisions; two existing GOLD records are separate</x:v>
+      </x:c>
+      <x:c r="D26" s="52"/>
+      <x:c r="E26" s="52"/>
+      <x:c r="F26" s="52"/>
+      <x:c r="G26" s="52"/>
+      <x:c r="H26" s="52"/>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="52" t="str">
+        <x:v>Include Yes</x:v>
+      </x:c>
+      <x:c r="B27" s="55" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C27" s="52" t="str">
+        <x:v>Newly adjudicated publications</x:v>
+      </x:c>
+      <x:c r="D27" s="52"/>
+      <x:c r="E27" s="52"/>
+      <x:c r="F27" s="52"/>
+      <x:c r="G27" s="52"/>
+      <x:c r="H27" s="52"/>
+    </x:row>
+    <x:row r="28" ht="42" customHeight="1">
+      <x:c r="A28" s="52" t="str">
+        <x:v>Include No</x:v>
+      </x:c>
+      <x:c r="B28" s="55" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C28" s="52" t="str">
+        <x:v>Newly adjudicated publications</x:v>
+      </x:c>
+      <x:c r="D28" s="52"/>
+      <x:c r="E28" s="52"/>
+      <x:c r="F28" s="52"/>
+      <x:c r="G28" s="52"/>
+      <x:c r="H28" s="52"/>
+    </x:row>
+    <x:row r="29" ht="42" customHeight="1">
+      <x:c r="A29" s="52" t="str">
+        <x:v>Publication inclusion yield</x:v>
+      </x:c>
+      <x:c r="B29" s="53" t="n">
+        <x:f>B27/B26</x:f>
+        <x:v>0.3888888888888889</x:v>
+      </x:c>
+      <x:c r="C29" s="52" t="str">
+        <x:v>7/18 among newly adjudicated publications</x:v>
+      </x:c>
+      <x:c r="D29" s="52"/>
+      <x:c r="E29" s="52"/>
+      <x:c r="F29" s="52"/>
+      <x:c r="G29" s="52"/>
+      <x:c r="H29" s="52"/>
+    </x:row>
+    <x:row r="30" ht="42" customHeight="1">
+      <x:c r="A30" s="52" t="str">
+        <x:v>New analyst report groups</x:v>
+      </x:c>
+      <x:c r="B30" s="55" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C30" s="52" t="str">
+        <x:v>Three pairs grouped for client-report purposes; Questel IDs retained</x:v>
+      </x:c>
+      <x:c r="D30" s="52"/>
+      <x:c r="E30" s="52"/>
+      <x:c r="F30" s="52"/>
+      <x:c r="G30" s="52"/>
+      <x:c r="H30" s="52"/>
+    </x:row>
+    <x:row r="31" ht="42" customHeight="1">
+      <x:c r="A31" s="52" t="str">
+        <x:v>Includable new candidate groups</x:v>
+      </x:c>
+      <x:c r="B31" s="55" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C31" s="52" t="str">
+        <x:v>Candidate groups; not established net-new relevant families</x:v>
+      </x:c>
+      <x:c r="D31" s="52"/>
+      <x:c r="E31" s="52"/>
+      <x:c r="F31" s="52"/>
+      <x:c r="G31" s="52"/>
+      <x:c r="H31" s="52"/>
+    </x:row>
+    <x:row r="32" ht="42" customHeight="1">
+      <x:c r="A32" s="52" t="str">
+        <x:v>Excluded new candidate groups</x:v>
+      </x:c>
+      <x:c r="B32" s="55" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C32" s="52" t="str">
+        <x:v>Analyst report-family grouping</x:v>
+      </x:c>
+      <x:c r="D32" s="52"/>
+      <x:c r="E32" s="52"/>
+      <x:c r="F32" s="52"/>
+      <x:c r="G32" s="52"/>
+      <x:c r="H32" s="52"/>
+    </x:row>
+    <x:row r="33" ht="42" customHeight="1">
+      <x:c r="A33" s="52" t="str">
+        <x:v>New-candidate family yield</x:v>
+      </x:c>
+      <x:c r="B33" s="53" t="n">
+        <x:f>B31/B30</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="C33" s="52" t="str">
+        <x:v>5/15 analyst-defined groups</x:v>
+      </x:c>
+      <x:c r="D33" s="52"/>
+      <x:c r="E33" s="52"/>
+      <x:c r="F33" s="52"/>
+      <x:c r="G33" s="52"/>
+      <x:c r="H33" s="52"/>
+    </x:row>
+    <x:row r="34" ht="42" customHeight="1">
+      <x:c r="A34" s="52" t="str">
+        <x:v>Top-20 publications evaluated</x:v>
+      </x:c>
+      <x:c r="B34" s="55" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C34" s="52" t="str">
+        <x:v>18 completed decisions plus two existing GOLD positives</x:v>
+      </x:c>
+      <x:c r="D34" s="52"/>
+      <x:c r="E34" s="52"/>
+      <x:c r="F34" s="52"/>
+      <x:c r="G34" s="52"/>
+      <x:c r="H34" s="52"/>
+    </x:row>
+    <x:row r="35" ht="42" customHeight="1">
+      <x:c r="A35" s="52" t="str">
+        <x:v>Top-20 positive publications</x:v>
+      </x:c>
+      <x:c r="B35" s="55" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C35" s="52" t="str">
+        <x:v>Includes the two existing GOLD records</x:v>
+      </x:c>
+      <x:c r="D35" s="52"/>
+      <x:c r="E35" s="52"/>
+      <x:c r="F35" s="52"/>
+      <x:c r="G35" s="52"/>
+      <x:c r="H35" s="52"/>
+    </x:row>
+    <x:row r="36" ht="42" customHeight="1">
+      <x:c r="A36" s="52" t="str">
+        <x:v>Publication Precision@20</x:v>
+      </x:c>
+      <x:c r="B36" s="54" t="n">
+        <x:f>B35/B34</x:f>
+        <x:v>0.45</x:v>
+      </x:c>
+      <x:c r="C36" s="52" t="str">
+        <x:v>9/20 original ranked records; not Questel-family precision</x:v>
+      </x:c>
+      <x:c r="D36" s="52"/>
+      <x:c r="E36" s="52"/>
+      <x:c r="F36" s="52"/>
+      <x:c r="G36" s="52"/>
+      <x:c r="H36" s="52"/>
+    </x:row>
+    <x:row r="37" ht="42" customHeight="1">
+      <x:c r="A37" s="52" t="str">
+        <x:v>Top-20 analyst report groups</x:v>
+      </x:c>
+      <x:c r="B37" s="55" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C37" s="52" t="str">
+        <x:v>No source rows or Questel identifiers merged</x:v>
+      </x:c>
+      <x:c r="D37" s="52"/>
+      <x:c r="E37" s="52"/>
+      <x:c r="F37" s="52"/>
+      <x:c r="G37" s="52"/>
+      <x:c r="H37" s="52"/>
+    </x:row>
+    <x:row r="38" ht="42" customHeight="1">
+      <x:c r="A38" s="52" t="str">
+        <x:v>Includable top-20 groups</x:v>
+      </x:c>
+      <x:c r="B38" s="55" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C38" s="52" t="str">
+        <x:v>Analyst report-family grouping</x:v>
+      </x:c>
+      <x:c r="D38" s="52"/>
+      <x:c r="E38" s="52"/>
+      <x:c r="F38" s="52"/>
+      <x:c r="G38" s="52"/>
+      <x:c r="H38" s="52"/>
+    </x:row>
+    <x:row r="39" ht="42" customHeight="1">
+      <x:c r="A39" s="52" t="str">
+        <x:v>Excluded top-20 groups</x:v>
+      </x:c>
+      <x:c r="B39" s="55" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C39" s="52" t="str">
+        <x:v>Analyst report-family grouping</x:v>
+      </x:c>
+      <x:c r="D39" s="52"/>
+      <x:c r="E39" s="52"/>
+      <x:c r="F39" s="52"/>
+      <x:c r="G39" s="52"/>
+      <x:c r="H39" s="52"/>
+    </x:row>
+    <x:row r="40" ht="42" customHeight="1">
+      <x:c r="A40" s="52" t="str">
+        <x:v>Report-inclusion yield@20</x:v>
+      </x:c>
+      <x:c r="B40" s="53" t="n">
+        <x:f>B38/B37</x:f>
+        <x:v>0.4117647058823529</x:v>
+      </x:c>
+      <x:c r="C40" s="52" t="str">
+        <x:v>7/17 family-deduplicated analyst report groups</x:v>
+      </x:c>
+      <x:c r="D40" s="52"/>
+      <x:c r="E40" s="52"/>
+      <x:c r="F40" s="52"/>
+      <x:c r="G40" s="52"/>
+      <x:c r="H40" s="52"/>
+    </x:row>
+    <x:row r="41" ht="42" customHeight="1">
+      <x:c r="A41" s="52" t="str">
+        <x:v>Net-new relevant-family yield</x:v>
+      </x:c>
+      <x:c r="B41" s="55" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="C41" s="52" t="str">
+        <x:v>Complete historical-report comparison pending</x:v>
+      </x:c>
+      <x:c r="D41" s="52"/>
+      <x:c r="E41" s="52"/>
+      <x:c r="F41" s="52"/>
+      <x:c r="G41" s="52"/>
+      <x:c r="H41" s="52"/>
+    </x:row>
+    <x:row r="42" ht="42" customHeight="1">
+      <x:c r="A42" s="52" t="str">
+        <x:v>Analyst review minutes</x:v>
+      </x:c>
+      <x:c r="B42" s="55" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="C42" s="52" t="str">
+        <x:v>Until supplied</x:v>
+      </x:c>
+      <x:c r="D42" s="52"/>
+      <x:c r="E42" s="52"/>
+      <x:c r="F42" s="52"/>
+      <x:c r="G42" s="52"/>
+      <x:c r="H42" s="52"/>
+    </x:row>
+    <x:row r="43" ht="42" customHeight="1">
+      <x:c r="A43" s="52" t="str">
+        <x:v>PA-001 status</x:v>
+      </x:c>
+      <x:c r="B43" s="55" t="str">
+        <x:v>COMPLETED</x:v>
+      </x:c>
+      <x:c r="C43" s="52" t="str">
+        <x:v>KZ6216U decision is abstract-only; not a claim of full-text availability</x:v>
+      </x:c>
+      <x:c r="D43" s="52"/>
+      <x:c r="E43" s="52"/>
+      <x:c r="F43" s="52"/>
+      <x:c r="G43" s="52"/>
+      <x:c r="H43" s="52"/>
+    </x:row>
+    <x:row r="44" ht="42" customHeight="1">
+      <x:c r="A44" s="52" t="str">
+        <x:v>Reconstructed mapping</x:v>
+      </x:c>
+      <x:c r="B44" s="55" t="str">
+        <x:v>Ambiguity retained</x:v>
+      </x:c>
+      <x:c r="C44" s="52" t="str">
+        <x:v>Ranks 6/7 remain unordered; same L/No decisions; no metric effect</x:v>
+      </x:c>
+      <x:c r="D44" s="52"/>
+      <x:c r="E44" s="52"/>
+      <x:c r="F44" s="52"/>
+      <x:c r="G44" s="52"/>
+      <x:c r="H44" s="52"/>
+    </x:row>
+    <x:row r="45" ht="42" customHeight="1">
+      <x:c r="A45" s="52" t="str">
+        <x:v>EXP-013 decision</x:v>
+      </x:c>
+      <x:c r="B45" s="55" t="str">
+        <x:v>HOLD / INCONCLUSIVE</x:v>
+      </x:c>
+      <x:c r="C45" s="52" t="str">
+        <x:v>V0 top 20 lacks equivalent adjudication; no promotion</x:v>
+      </x:c>
+      <x:c r="D45" s="52"/>
+      <x:c r="E45" s="52"/>
+      <x:c r="F45" s="52"/>
+      <x:c r="G45" s="52"/>
+      <x:c r="H45" s="52"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
     <x:mergeCell ref="A12:H12"/>
     <x:mergeCell ref="A13:H17"/>
     <x:mergeCell ref="A19:H19"/>
+    <x:mergeCell ref="C25:H25"/>
+    <x:mergeCell ref="C26:H26"/>
+    <x:mergeCell ref="C27:H27"/>
+    <x:mergeCell ref="C28:H28"/>
+    <x:mergeCell ref="C29:H29"/>
+    <x:mergeCell ref="C30:H30"/>
+    <x:mergeCell ref="C31:H31"/>
+    <x:mergeCell ref="C32:H32"/>
+    <x:mergeCell ref="C33:H33"/>
+    <x:mergeCell ref="C34:H34"/>
+    <x:mergeCell ref="C35:H35"/>
+    <x:mergeCell ref="C36:H36"/>
+    <x:mergeCell ref="C37:H37"/>
+    <x:mergeCell ref="C38:H38"/>
+    <x:mergeCell ref="C39:H39"/>
+    <x:mergeCell ref="C40:H40"/>
+    <x:mergeCell ref="C41:H41"/>
+    <x:mergeCell ref="C42:H42"/>
+    <x:mergeCell ref="C43:H43"/>
+    <x:mergeCell ref="C44:H44"/>
+    <x:mergeCell ref="C45:H45"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1586,7 +1982,7 @@
         <x:v>Current V0 retrieval baseline</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="300" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:v>EXP-013</x:v>
       </x:c>
@@ -1626,15 +2022,19 @@
       <x:c r="M16" s="31" t="n">
         <x:v>0.4</x:v>
       </x:c>
-      <x:c r="N16" s="31"/>
+      <x:c r="N16" s="51" t="n">
+        <x:v>0.45</x:v>
+      </x:c>
       <x:c r="O16" s="24"/>
       <x:c r="P16" s="43" t="n">
         <x:v>90.5</x:v>
       </x:c>
-      <x:c r="Q16" s="44"/>
+      <x:c r="Q16" s="44" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
       <x:c r="R16" s="32"/>
       <x:c r="S16" s="24" t="str">
-        <x:v>18/20 top families unjudged; title/abstract only</x:v>
+        <x:v>V0 top 20 not equivalently adjudicated; three analyst report-family pairs have different Questel FAN IDs; theft-triggered locking schema review pending</x:v>
       </x:c>
       <x:c r="T16" s="24" t="str">
         <x:v>Recall@100 2/10→4/10; median retrieved-GOLD rank 492→90.5</x:v>
@@ -1643,7 +2043,7 @@
         <x:v>HOLD</x:v>
       </x:c>
       <x:c r="V16" s="24" t="str">
-        <x:v>INCONCLUSIVE pending top-20 adjudication</x:v>
+        <x:v>PA-001 COMPLETED. HOLD / INCONCLUSIVE: V0 top 20 lacks equivalent adjudication. Newly adjudicated: 18 (7 Yes, 11 No), inclusion 7/18 = 38.9%. Publication Precision@20 incl. 2 GOLD: 9/20 = 45%. New analyst report groups: 15 (5 included, 10 excluded), yield 5/15 = 33.3%. Top-20 analyst report groups: 17 (7 included, 10 excluded), report-inclusion yield 7/17 = 41.2%. Net-new relevant-family yield and analyst minutes: N/A. Reconstructed mapping; unordered ranks 6/7 L/No ambiguity has no metric effect. No promotion.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -6110,7 +6510,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68b2f64743ea4b2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b9397289ba147ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6473,27 +6873,27 @@
         <x:v>Improved from 492</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="65" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:v>Pending Validation</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
-        <x:v>V1 top-20 unjudged families</x:v>
+        <x:v>V1 top-20 adjudication</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
         <x:v>PA-001</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
-        <x:v>BLOCKING</x:v>
+        <x:v>COMPLETED</x:v>
       </x:c>
       <x:c r="E16" s="24" t="n">
-        <x:v>18</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F16" s="24" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="G16" s="24" t="str">
-        <x:v>Needed for true Precision@20 and net-new relevant yield</x:v>
+        <x:v>PA-001 completed: 18 analyst decisions + 2 GOLD. V0 comparative adjudication and net-new report comparison remain outstanding.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -6847,7 +7247,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbb46d22c1e44b7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20c02993f3cb4a1c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6980,7 +7380,7 @@
         <x:v>Single query; 6/10 GOLD; 4 GOLD absent; live database changes</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="90" customHeight="1">
       <x:c r="A6" s="24" t="str">
         <x:v>Relevance Scorer</x:v>
       </x:c>
@@ -6988,7 +7388,7 @@
         <x:v>rs_v0.2_blind_ta_rerank</x:v>
       </x:c>
       <x:c r="C6" s="24" t="str">
-        <x:v>Metrics computed; practical precision pending</x:v>
+        <x:v>HOLD / INCONCLUSIVE</x:v>
       </x:c>
       <x:c r="D6" s="24" t="str">
         <x:v>Rank retrieved families</x:v>
@@ -7000,7 +7400,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G6" s="24" t="str">
-        <x:v>Title/abstract only; model/version not frozen; top-20 mostly unjudged; label calibration weak</x:v>
+        <x:v>V1 top 20 adjudicated; V0 comparison pending; three report-family groups differ from Questel IDs; model/version and label calibration limitations remain</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -7250,7 +7650,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra62700ed683a417a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c61a544150849d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7334,21 +7734,21 @@
         <x:v>V0 2/10; V1 4/10</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="80" customHeight="1">
       <x:c r="A5" s="24" t="str">
-        <x:v>Precision@20</x:v>
+        <x:v>Publication Precision@20</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
-        <x:v>Analyst-relevant families among first 20 / 20</x:v>
+        <x:v>Analyst-positive publications among original V1 top 20 / 20; includes two existing GOLD positives</x:v>
       </x:c>
       <x:c r="C5" s="24" t="str">
         <x:v>Measures practical usefulness of top results</x:v>
       </x:c>
       <x:c r="D5" s="24" t="str">
-        <x:v>All top-20 records adjudicated</x:v>
+        <x:v>All top-20 outcomes evaluated; identical-content ambiguity must not affect outcomes</x:v>
       </x:c>
       <x:c r="E5" s="24" t="str">
-        <x:v>PENDING — 18/20 V1 families unjudged</x:v>
+        <x:v>EXP-013: 9/20 = 45%; PA-001 COMPLETED; HOLD pending V0 comparison</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -7402,12 +7802,22 @@
         <x:v>~30 min → 10–15 min on 5-patent sample</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="24"/>
-      <x:c r="B9" s="24"/>
-      <x:c r="C9" s="24"/>
-      <x:c r="D9" s="24"/>
-      <x:c r="E9" s="24"/>
+    <x:row r="9" ht="95" customHeight="1">
+      <x:c r="A9" s="24" t="str">
+        <x:v>Family-deduplicated report-inclusion yield@20</x:v>
+      </x:c>
+      <x:c r="B9" s="24" t="str">
+        <x:v>Includable analyst-defined report groups among top-20 records / all analyst-defined report groups</x:v>
+      </x:c>
+      <x:c r="C9" s="24" t="str">
+        <x:v>Separates client-report grouping from publication precision</x:v>
+      </x:c>
+      <x:c r="D9" s="24" t="str">
+        <x:v>Explicit analyst grouping; Questel IDs retained</x:v>
+      </x:c>
+      <x:c r="E9" s="24" t="str">
+        <x:v>EXP-013: 7/17 = 41.2%; not a Questel-family precision estimate</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="24"/>
@@ -7559,7 +7969,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45e20ee4ac5649b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb30d0148fdb44d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Set up EXP-014 Orbit versus AI top-20 comparison
</commit_message>
<xml_diff>
--- a/Patent_AI_Experiment_Dashboard_Canonical.xlsx
+++ b/Patent_AI_Experiment_Dashboard_Canonical.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R518a98c7c2e74836"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" r:id="Rbd23c3c2892147f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Inputs" sheetId="3" r:id="R1147256ed16e40e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Versions" sheetId="4" r:id="Rce7c9615e51c4fd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Definitions" sheetId="5" r:id="R460990d3bb2646d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6335235a76a54e53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" r:id="Rf15bf277183144aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Inputs" sheetId="3" r:id="R8f1ef3d204704bbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Versions" sheetId="4" r:id="R21cf4aa0f9ec41c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Definitions" sheetId="5" r:id="R3cbade6532cc4f98"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -49,7 +49,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -86,6 +86,11 @@
         <x:fgColor rgb="FF4472C4"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -94,7 +99,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="58">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -211,6 +216,8 @@
     <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -594,7 +601,7 @@
       </x:c>
       <x:c r="E5" t="n">
         <x:f>COUNTA('Experiment Log'!A2:A200)</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -632,7 +639,7 @@
         <x:v>Current Experiment</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>EXP-013</x:v>
+        <x:v>EXP-014</x:v>
       </x:c>
       <x:c r="D8" t="str">
         <x:v>Best Recall@100</x:v>
@@ -1175,6 +1182,354 @@
       <x:c r="F45" s="52"/>
       <x:c r="G45" s="52"/>
       <x:c r="H45" s="52"/>
+    </x:row>
+    <x:row r="48" ht="32" customHeight="1">
+      <x:c r="A48" s="59" t="str">
+        <x:v>EXP-014 — Orbit versus frozen AI top-20 comparison</x:v>
+      </x:c>
+      <x:c r="B48" s="59"/>
+      <x:c r="C48" s="59"/>
+      <x:c r="D48" s="59"/>
+      <x:c r="E48" s="59"/>
+      <x:c r="F48" s="59"/>
+      <x:c r="G48" s="59"/>
+      <x:c r="H48" s="59"/>
+    </x:row>
+    <x:row r="49" ht="50" customHeight="1">
+      <x:c r="A49" s="52" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="B49" s="52" t="str">
+        <x:v>AWAITING_ADJUDICATION</x:v>
+      </x:c>
+      <x:c r="C49" s="52" t="str">
+        <x:v>Setup only; no final evaluation decision</x:v>
+      </x:c>
+      <x:c r="D49" s="52"/>
+      <x:c r="E49" s="52"/>
+      <x:c r="F49" s="52"/>
+      <x:c r="G49" s="52"/>
+      <x:c r="H49" s="52"/>
+    </x:row>
+    <x:row r="50" ht="50" customHeight="1">
+      <x:c r="A50" s="52" t="str">
+        <x:v>Baseline</x:v>
+      </x:c>
+      <x:c r="B50" s="52" t="str">
+        <x:v>RUN-012 Orbit ordering</x:v>
+      </x:c>
+      <x:c r="C50" s="52" t="str">
+        <x:v>Same frozen 3,238-family export</x:v>
+      </x:c>
+      <x:c r="D50" s="52"/>
+      <x:c r="E50" s="52"/>
+      <x:c r="F50" s="52"/>
+      <x:c r="G50" s="52"/>
+      <x:c r="H50" s="52"/>
+    </x:row>
+    <x:row r="51" ht="50" customHeight="1">
+      <x:c r="A51" s="52" t="str">
+        <x:v>Challenger</x:v>
+      </x:c>
+      <x:c r="B51" s="52" t="str">
+        <x:v>rs_v0.2_blind_ta_rerank</x:v>
+      </x:c>
+      <x:c r="C51" s="52" t="str">
+        <x:v>Frozen EXP-013 ranking</x:v>
+      </x:c>
+      <x:c r="D51" s="52"/>
+      <x:c r="E51" s="52"/>
+      <x:c r="F51" s="52"/>
+      <x:c r="G51" s="52"/>
+      <x:c r="H51" s="52"/>
+    </x:row>
+    <x:row r="52" ht="50" customHeight="1">
+      <x:c r="A52" s="52" t="str">
+        <x:v>Component evaluated</x:v>
+      </x:c>
+      <x:c r="B52" s="52" t="str">
+        <x:v>Relevance Scorer</x:v>
+      </x:c>
+      <x:c r="C52" s="52" t="str">
+        <x:v>Ranking evaluation; no model or system change</x:v>
+      </x:c>
+      <x:c r="D52" s="52"/>
+      <x:c r="E52" s="52"/>
+      <x:c r="F52" s="52"/>
+      <x:c r="G52" s="52"/>
+      <x:c r="H52" s="52"/>
+    </x:row>
+    <x:row r="53" ht="50" customHeight="1">
+      <x:c r="A53" s="52" t="str">
+        <x:v>Single primary change</x:v>
+      </x:c>
+      <x:c r="B53" s="52" t="str">
+        <x:v>ordering method</x:v>
+      </x:c>
+      <x:c r="C53" s="52" t="str">
+        <x:v>Disclosure, benchmark, universe, query/database, relevance standard, ground truth, rankings and family policy fixed</x:v>
+      </x:c>
+      <x:c r="D53" s="52"/>
+      <x:c r="E53" s="52"/>
+      <x:c r="F53" s="52"/>
+      <x:c r="G53" s="52"/>
+      <x:c r="H53" s="52"/>
+    </x:row>
+    <x:row r="54" ht="50" customHeight="1">
+      <x:c r="A54" s="52" t="str">
+        <x:v>Hypothesis</x:v>
+      </x:c>
+      <x:c r="B54" s="52" t="str">
+        <x:v>At least 2 more includable groups</x:v>
+      </x:c>
+      <x:c r="C54" s="52" t="str">
+        <x:v>V1 finds at least two more includable unique report-family groups in the first 20 publication slots and passes both recall guardrails</x:v>
+      </x:c>
+      <x:c r="D54" s="52"/>
+      <x:c r="E54" s="52"/>
+      <x:c r="F54" s="52"/>
+      <x:c r="G54" s="52"/>
+      <x:c r="H54" s="52"/>
+    </x:row>
+    <x:row r="55" ht="50" customHeight="1">
+      <x:c r="A55" s="52" t="str">
+        <x:v>Resolved publications</x:v>
+      </x:c>
+      <x:c r="B55" s="52" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C55" s="52" t="str">
+        <x:v>Existing decisions: WO2021194584A2 family H/Yes; CN207144670U L/No</x:v>
+      </x:c>
+      <x:c r="D55" s="52"/>
+      <x:c r="E55" s="52"/>
+      <x:c r="F55" s="52"/>
+      <x:c r="G55" s="52"/>
+      <x:c r="H55" s="52"/>
+    </x:row>
+    <x:row r="56" ht="50" customHeight="1">
+      <x:c r="A56" s="52" t="str">
+        <x:v>Unresolved publications</x:v>
+      </x:c>
+      <x:c r="B56" s="52" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C56" s="52" t="str">
+        <x:v>Shuffled analyst packet; no inferred labels</x:v>
+      </x:c>
+      <x:c r="D56" s="52"/>
+      <x:c r="E56" s="52"/>
+      <x:c r="F56" s="52"/>
+      <x:c r="G56" s="52"/>
+      <x:c r="H56" s="52"/>
+    </x:row>
+    <x:row r="57" ht="50" customHeight="1">
+      <x:c r="A57" s="52" t="str">
+        <x:v>Top-20 publication overlap</x:v>
+      </x:c>
+      <x:c r="B57" s="52" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C57" s="52" t="str">
+        <x:v>CN207144670U; Questel FAN overlap also one</x:v>
+      </x:c>
+      <x:c r="D57" s="52"/>
+      <x:c r="E57" s="52"/>
+      <x:c r="F57" s="52"/>
+      <x:c r="G57" s="52"/>
+      <x:c r="H57" s="52"/>
+    </x:row>
+    <x:row r="58" ht="50" customHeight="1">
+      <x:c r="A58" s="52" t="str">
+        <x:v>Known report groups</x:v>
+      </x:c>
+      <x:c r="B58" s="52" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C58" s="52" t="str">
+        <x:v>One includable, one excluded; unresolved families remain unassigned</x:v>
+      </x:c>
+      <x:c r="D58" s="52"/>
+      <x:c r="E58" s="52"/>
+      <x:c r="F58" s="52"/>
+      <x:c r="G58" s="52"/>
+      <x:c r="H58" s="52"/>
+    </x:row>
+    <x:row r="59" ht="50" customHeight="1">
+      <x:c r="A59" s="52" t="str">
+        <x:v>Primary metric: V0 includable groups</x:v>
+      </x:c>
+      <x:c r="B59" s="52" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="C59" s="52" t="str">
+        <x:v>Number of analyst-includable unique report-family groups in first 20 publication slots</x:v>
+      </x:c>
+      <x:c r="D59" s="52"/>
+      <x:c r="E59" s="52"/>
+      <x:c r="F59" s="52"/>
+      <x:c r="G59" s="52"/>
+      <x:c r="H59" s="52"/>
+    </x:row>
+    <x:row r="60" ht="50" customHeight="1">
+      <x:c r="A60" s="52" t="str">
+        <x:v>V0 publication Precision@20</x:v>
+      </x:c>
+      <x:c r="B60" s="52" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="C60" s="52" t="str">
+        <x:v>Pending complete adjudication</x:v>
+      </x:c>
+      <x:c r="D60" s="52"/>
+      <x:c r="E60" s="52"/>
+      <x:c r="F60" s="52"/>
+      <x:c r="G60" s="52"/>
+      <x:c r="H60" s="52"/>
+    </x:row>
+    <x:row r="61" ht="50" customHeight="1">
+      <x:c r="A61" s="52" t="str">
+        <x:v>V0 report-family inclusion yield</x:v>
+      </x:c>
+      <x:c r="B61" s="52" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="C61" s="52" t="str">
+        <x:v>Pending complete adjudication and group reconciliation</x:v>
+      </x:c>
+      <x:c r="D61" s="52"/>
+      <x:c r="E61" s="52"/>
+      <x:c r="F61" s="52"/>
+      <x:c r="G61" s="52"/>
+      <x:c r="H61" s="52"/>
+    </x:row>
+    <x:row r="62" ht="50" customHeight="1">
+      <x:c r="A62" s="52" t="str">
+        <x:v>Analyst review minutes</x:v>
+      </x:c>
+      <x:c r="B62" s="52" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="C62" s="52" t="str">
+        <x:v>One total active time requested; access delays excluded</x:v>
+      </x:c>
+      <x:c r="D62" s="52"/>
+      <x:c r="E62" s="52"/>
+      <x:c r="F62" s="52"/>
+      <x:c r="G62" s="52"/>
+      <x:c r="H62" s="52"/>
+    </x:row>
+    <x:row r="63" ht="50" customHeight="1">
+      <x:c r="A63" s="52" t="str">
+        <x:v>Recall@50 guardrail</x:v>
+      </x:c>
+      <x:c r="B63" s="52" t="str">
+        <x:v>Pass (frozen metrics)</x:v>
+      </x:c>
+      <x:c r="C63" s="52" t="str">
+        <x:v>V1 2/10 &gt;= V0 2/10; no new run</x:v>
+      </x:c>
+      <x:c r="D63" s="52"/>
+      <x:c r="E63" s="52"/>
+      <x:c r="F63" s="52"/>
+      <x:c r="G63" s="52"/>
+      <x:c r="H63" s="52"/>
+    </x:row>
+    <x:row r="64" ht="50" customHeight="1">
+      <x:c r="A64" s="52" t="str">
+        <x:v>Recall@100 guardrail</x:v>
+      </x:c>
+      <x:c r="B64" s="52" t="str">
+        <x:v>Pass (frozen metrics)</x:v>
+      </x:c>
+      <x:c r="C64" s="52" t="str">
+        <x:v>V1 4/10 &gt; V0 2/10; no new run</x:v>
+      </x:c>
+      <x:c r="D64" s="52"/>
+      <x:c r="E64" s="52"/>
+      <x:c r="F64" s="52"/>
+      <x:c r="G64" s="52"/>
+      <x:c r="H64" s="52"/>
+    </x:row>
+    <x:row r="65" ht="50" customHeight="1">
+      <x:c r="A65" s="52" t="str">
+        <x:v>Final EXP-014 decision</x:v>
+      </x:c>
+      <x:c r="B65" s="52" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="C65" s="52" t="str">
+        <x:v>No PROMOTE / REJECT / HOLD outcome calculated</x:v>
+      </x:c>
+      <x:c r="D65" s="52"/>
+      <x:c r="E65" s="52"/>
+      <x:c r="F65" s="52"/>
+      <x:c r="G65" s="52"/>
+      <x:c r="H65" s="52"/>
+    </x:row>
+    <x:row r="66" ht="50" customHeight="1">
+      <x:c r="A66" s="52" t="str">
+        <x:v>Pre-registered PROMOTE</x:v>
+      </x:c>
+      <x:c r="B66" s="52" t="str">
+        <x:v>V1 at least 2 groups better</x:v>
+      </x:c>
+      <x:c r="C66" s="52" t="str">
+        <x:v>Requires both recall guardrails to pass</x:v>
+      </x:c>
+      <x:c r="D66" s="52"/>
+      <x:c r="E66" s="52"/>
+      <x:c r="F66" s="52"/>
+      <x:c r="G66" s="52"/>
+      <x:c r="H66" s="52"/>
+    </x:row>
+    <x:row r="67" ht="50" customHeight="1">
+      <x:c r="A67" s="52" t="str">
+        <x:v>Pre-registered REJECT</x:v>
+      </x:c>
+      <x:c r="B67" s="52" t="str">
+        <x:v>V1 fewer groups OR guardrail failure</x:v>
+      </x:c>
+      <x:c r="C67" s="52" t="str">
+        <x:v>Guardrail failure takes precedence over group-count HOLD condition</x:v>
+      </x:c>
+      <x:c r="D67" s="52"/>
+      <x:c r="E67" s="52"/>
+      <x:c r="F67" s="52"/>
+      <x:c r="G67" s="52"/>
+      <x:c r="H67" s="52"/>
+    </x:row>
+    <x:row r="68" ht="50" customHeight="1">
+      <x:c r="A68" s="52" t="str">
+        <x:v>Pre-registered HOLD</x:v>
+      </x:c>
+      <x:c r="B68" s="52" t="str">
+        <x:v>Equal or 1 group better</x:v>
+      </x:c>
+      <x:c r="C68" s="52" t="str">
+        <x:v>With both recall guardrails passing</x:v>
+      </x:c>
+      <x:c r="D68" s="52"/>
+      <x:c r="E68" s="52"/>
+      <x:c r="F68" s="52"/>
+      <x:c r="G68" s="52"/>
+      <x:c r="H68" s="52"/>
+    </x:row>
+    <x:row r="69" ht="50" customHeight="1">
+      <x:c r="A69" s="52" t="str">
+        <x:v>Final V0 report-group denominator</x:v>
+      </x:c>
+      <x:c r="B69" s="52" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="C69" s="52" t="str">
+        <x:v>Two groups currently identifiable; do not assume all other records are separate families</x:v>
+      </x:c>
+      <x:c r="D69" s="52"/>
+      <x:c r="E69" s="52"/>
+      <x:c r="F69" s="52"/>
+      <x:c r="G69" s="52"/>
+      <x:c r="H69" s="52"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1203,6 +1558,28 @@
     <x:mergeCell ref="C43:H43"/>
     <x:mergeCell ref="C44:H44"/>
     <x:mergeCell ref="C45:H45"/>
+    <x:mergeCell ref="A48:H48"/>
+    <x:mergeCell ref="C49:H49"/>
+    <x:mergeCell ref="C50:H50"/>
+    <x:mergeCell ref="C51:H51"/>
+    <x:mergeCell ref="C52:H52"/>
+    <x:mergeCell ref="C53:H53"/>
+    <x:mergeCell ref="C54:H54"/>
+    <x:mergeCell ref="C55:H55"/>
+    <x:mergeCell ref="C56:H56"/>
+    <x:mergeCell ref="C57:H57"/>
+    <x:mergeCell ref="C58:H58"/>
+    <x:mergeCell ref="C59:H59"/>
+    <x:mergeCell ref="C60:H60"/>
+    <x:mergeCell ref="C61:H61"/>
+    <x:mergeCell ref="C62:H62"/>
+    <x:mergeCell ref="C63:H63"/>
+    <x:mergeCell ref="C64:H64"/>
+    <x:mergeCell ref="C65:H65"/>
+    <x:mergeCell ref="C66:H66"/>
+    <x:mergeCell ref="C67:H67"/>
+    <x:mergeCell ref="C68:H68"/>
+    <x:mergeCell ref="C69:H69"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2046,29 +2423,73 @@
         <x:v>PA-001 COMPLETED. HOLD / INCONCLUSIVE: V0 top 20 lacks equivalent adjudication. Newly adjudicated: 18 (7 Yes, 11 No), inclusion 7/18 = 38.9%. Publication Precision@20 incl. 2 GOLD: 9/20 = 45%. New analyst report groups: 15 (5 included, 10 excluded), yield 5/15 = 33.3%. Top-20 analyst report groups: 17 (7 included, 10 excluded), report-inclusion yield 7/17 = 41.2%. Net-new relevant-family yield and analyst minutes: N/A. Reconstructed mapping; unordered ranks 6/7 L/No ambiguity has no metric effect. No promotion.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="24"/>
-      <x:c r="B17" s="30"/>
-      <x:c r="C17" s="24"/>
-      <x:c r="D17" s="24"/>
-      <x:c r="E17" s="24"/>
-      <x:c r="F17" s="24"/>
-      <x:c r="G17" s="24"/>
-      <x:c r="H17" s="24"/>
-      <x:c r="I17" s="24"/>
-      <x:c r="J17" s="24"/>
-      <x:c r="K17" s="24"/>
-      <x:c r="L17" s="31"/>
-      <x:c r="M17" s="31"/>
-      <x:c r="N17" s="31"/>
-      <x:c r="O17" s="24"/>
-      <x:c r="P17" s="43"/>
-      <x:c r="Q17" s="44"/>
-      <x:c r="R17" s="32"/>
-      <x:c r="S17" s="24"/>
-      <x:c r="T17" s="24"/>
-      <x:c r="U17" s="24"/>
-      <x:c r="V17" s="24"/>
+    <x:row r="17" ht="300" customHeight="1">
+      <x:c r="A17" s="24" t="str">
+        <x:v>EXP-014</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="C17" s="24" t="str">
+        <x:v>BC001</x:v>
+      </x:c>
+      <x:c r="D17" s="24" t="str">
+        <x:v>0.1-provisional</x:v>
+      </x:c>
+      <x:c r="E17" s="24" t="str">
+        <x:v>RUN-012 Orbit ordering of the 3,238-family export</x:v>
+      </x:c>
+      <x:c r="F17" s="24" t="str">
+        <x:v>rs_v0.2_blind_ta_rerank</x:v>
+      </x:c>
+      <x:c r="G17" s="24" t="str">
+        <x:v>V1 finds at least two more analyst-includable unique report-family groups in the first 20 publication slots than V0 while passing both recall guardrails</x:v>
+      </x:c>
+      <x:c r="H17" s="24" t="str">
+        <x:v>Relevance Scorer</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="str">
+        <x:v>RUN-012 Orbit ordering</x:v>
+      </x:c>
+      <x:c r="J17" s="24" t="str">
+        <x:v>rs_v0.2_blind_ta_rerank (frozen EXP-013)</x:v>
+      </x:c>
+      <x:c r="K17" s="24" t="str">
+        <x:v>ordering method; ranking evaluation; no model or system change</x:v>
+      </x:c>
+      <x:c r="L17" s="31" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="M17" s="31" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N17" s="31" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="O17" s="24" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="P17" s="43" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="Q17" s="44" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="R17" s="32" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="S17" s="24" t="str">
+        <x:v>V1 Recall@50 &gt;= V0 Recall@50; V1 Recall@100 &gt; V0 Recall@100. All rankings, universe, ground truth and family policy fixed.</x:v>
+      </x:c>
+      <x:c r="T17" s="24" t="str">
+        <x:v>N/A pending adjudication</x:v>
+      </x:c>
+      <x:c r="U17" s="24" t="str">
+        <x:v>AWAITING_ADJUDICATION</x:v>
+      </x:c>
+      <x:c r="V17" s="24" t="str">
+        <x:v>PROMOTE if V1 has &gt;=2 more includable unique report-family groups and both recall guardrails pass; REJECT if V1 has fewer or violates either guardrail; HOLD if equal or one better (guardrails pass). 2 resolved, 18 unresolved; overlap 1; final metrics and review minutes N/A. No decision calculated.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="24"/>
@@ -6505,12 +6926,12 @@
       <x:formula1>"Human baseline,Feature Extractor,Terminology Engine,Query Planner,Retrieval Adapter,Relevance Scorer,Evidence Extractor,Search Controller,Evaluation,Multi-component"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="U2:U200">
-      <x:formula1>"BASELINE,DIAGNOSTIC,PARTIALLY_VALIDATED,HOLD,PROMOTE,REJECT,SUPERSEDED,INCONCLUSIVE"</x:formula1>
+      <x:formula1>"BASELINE,DIAGNOSTIC,PARTIALLY_VALIDATED,HOLD,PROMOTE,REJECT,SUPERSEDED,INCONCLUSIVE,AWAITING_ADJUDICATION"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b9397289ba147ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28254b7d60c74182"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7247,7 +7668,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20c02993f3cb4a1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7204510f3032472c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7650,7 +8071,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c61a544150849d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d4f23c1aeec4b57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7969,7 +8390,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb30d0148fdb44d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf75faaeeffe4e12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record EXP-016A scorer failure audit
</commit_message>
<xml_diff>
--- a/Patent_AI_Experiment_Dashboard_Canonical.xlsx
+++ b/Patent_AI_Experiment_Dashboard_Canonical.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5360d3d03b3f4da4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" r:id="R863412b69bd046d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Inputs" sheetId="3" r:id="R55933a9a84144a57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Versions" sheetId="4" r:id="R608d0ec7ce274400"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Definitions" sheetId="5" r:id="Re93b83cbb01c418e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf1dbbe9fc2c44a4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" r:id="Rbce225dc2fc94c43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Inputs" sheetId="3" r:id="R4aed6fdbebbe49fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Versions" sheetId="4" r:id="Rabb92be259e24cbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Definitions" sheetId="5" r:id="Rfbf8fc4337da4901"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1876,7 +1876,7 @@
     </x:row>
     <x:row r="98" ht="22" customHeight="1">
       <x:c r="A98" s="36" t="str">
-        <x:v>Deterministic rule extraction; evidence judgments are not analyst labels. Component remains a challenger.</x:v>
+        <x:v>D1: extractor semantics/domain boundaries failed; weights alone not established. EXP-018 proposed only; no rerank.</x:v>
       </x:c>
       <x:c r="B98" s="36"/>
       <x:c r="C98" s="36"/>
@@ -3002,13 +3002,13 @@
         <x:v>Recall@20 1/10 fails 2/10 guardrail; Recall@200 3/10; median worsens &gt;10%</x:v>
       </x:c>
       <x:c r="T19" s="52" t="str">
-        <x:v>Determinism did not improve retrieval ordering of known GOLD; rule extraction needs separate evaluation</x:v>
+        <x:v>D1: semantic extraction/gating errors in 3/3 deteriorated GOLD. Weight-only failure not established.</x:v>
       </x:c>
       <x:c r="U19" s="52" t="str">
         <x:v>REJECT</x:v>
       </x:c>
       <x:c r="V19" s="52" t="str">
-        <x:v>Frozen before private evaluation. Six GOLD mappings exact in reconstructed key. Challenger only; CURRENT_SYSTEM unchanged.</x:v>
+        <x:v>Post-hoc D1 audit; no rerank. Penalty/cap contribution 2/3; title/abstract limits 2/3 (overlapping). EXP-018 semantic extraction proposed only. REJECT unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -7403,7 +7403,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03e923d14b0a4565"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f8e6fa386ba449b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8140,7 +8140,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra05ca7f7fd1c48ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb71efb718c8c45f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8557,7 +8557,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R731516e309cf45a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6bea4489cbc45dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8876,7 +8876,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0fffed3cafd4114"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaf62b19a88a4e10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Set up EXP-017A proximity volume preflight
</commit_message>
<xml_diff>
--- a/Patent_AI_Experiment_Dashboard_Canonical.xlsx
+++ b/Patent_AI_Experiment_Dashboard_Canonical.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf1dbbe9fc2c44a4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" r:id="Rbce225dc2fc94c43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Inputs" sheetId="3" r:id="R4aed6fdbebbe49fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Versions" sheetId="4" r:id="Rabb92be259e24cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Definitions" sheetId="5" r:id="Rfbf8fc4337da4901"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb7a666564c424511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" r:id="R10c2a651947d4766"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Inputs" sheetId="3" r:id="R2beb5e573064478b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Versions" sheetId="4" r:id="R76426214d8914b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Definitions" sheetId="5" r:id="R9f1ee8d2393b442d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -50,7 +50,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -102,6 +102,11 @@
         <x:fgColor rgb="FF4472C4"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -110,7 +115,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="69">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -246,6 +251,12 @@
     <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="207" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -629,7 +640,7 @@
       </x:c>
       <x:c r="E5" t="n">
         <x:f>COUNTA('Experiment Log'!A2:A200)</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -667,7 +678,7 @@
         <x:v>Current Experiment</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>EXP-016A</x:v>
+        <x:v>EXP-017A</x:v>
       </x:c>
       <x:c r="D8" t="str">
         <x:v>Best Recall@100</x:v>
@@ -1897,6 +1908,138 @@
       <x:c r="F99" s="36"/>
       <x:c r="G99" s="36"/>
       <x:c r="H99" s="36"/>
+    </x:row>
+    <x:row r="110" ht="32" customHeight="1">
+      <x:c r="A110" s="70" t="str">
+        <x:v>EXP-017A — Proximity-based retrieval volume preflight</x:v>
+      </x:c>
+      <x:c r="B110" s="70"/>
+      <x:c r="C110" s="70"/>
+      <x:c r="D110" s="70"/>
+      <x:c r="E110" s="70"/>
+      <x:c r="F110" s="70"/>
+      <x:c r="G110" s="70"/>
+      <x:c r="H110" s="70"/>
+    </x:row>
+    <x:row r="111" ht="32" customHeight="1">
+      <x:c r="A111" s="69" t="str">
+        <x:v>AWAITING_ORBIT_PREFLIGHT</x:v>
+      </x:c>
+      <x:c r="B111" s="69"/>
+      <x:c r="C111" s="69"/>
+      <x:c r="D111" s="69"/>
+      <x:c r="E111" s="69"/>
+      <x:c r="F111" s="69"/>
+      <x:c r="G111" s="69"/>
+      <x:c r="H111" s="69"/>
+    </x:row>
+    <x:row r="112" ht="32" customHeight="1">
+      <x:c r="A112" s="24" t="str">
+        <x:v>Single change: cross-concept AND replaced with unordered 5D. Analyst execution pending.</x:v>
+      </x:c>
+      <x:c r="B112" s="24"/>
+      <x:c r="C112" s="24"/>
+      <x:c r="D112" s="24"/>
+      <x:c r="E112" s="24"/>
+      <x:c r="F112" s="24"/>
+      <x:c r="G112" s="24"/>
+      <x:c r="H112" s="24"/>
+    </x:row>
+    <x:row r="113" ht="32" customHeight="1">
+      <x:c r="A113" s="24" t="str">
+        <x:v>Q1P biometric/authentication: baseline 23,935 FAMPAT families. Proximity count: pending.</x:v>
+      </x:c>
+      <x:c r="B113" s="24"/>
+      <x:c r="C113" s="24"/>
+      <x:c r="D113" s="24"/>
+      <x:c r="E113" s="24"/>
+      <x:c r="F113" s="24"/>
+      <x:c r="G113" s="24"/>
+      <x:c r="H113" s="24"/>
+    </x:row>
+    <x:row r="114" ht="32" customHeight="1">
+      <x:c r="A114" s="24" t="str">
+        <x:v>Q2P locking/control: baseline 493,993 FAMPAT families. Proximity count: pending.</x:v>
+      </x:c>
+      <x:c r="B114" s="24"/>
+      <x:c r="C114" s="24"/>
+      <x:c r="D114" s="24"/>
+      <x:c r="E114" s="24"/>
+      <x:c r="F114" s="24"/>
+      <x:c r="G114" s="24"/>
+      <x:c r="H114" s="24"/>
+    </x:row>
+    <x:row r="115" ht="32" customHeight="1">
+      <x:c r="A115" s="24" t="str">
+        <x:v>Fixed: FAMPAT, TI/AB/CLMS, current vocabulary. No filters or expansion. No benchmark changes.</x:v>
+      </x:c>
+      <x:c r="B115" s="24"/>
+      <x:c r="C115" s="24"/>
+      <x:c r="D115" s="24"/>
+      <x:c r="E115" s="24"/>
+      <x:c r="F115" s="24"/>
+      <x:c r="G115" s="24"/>
+      <x:c r="H115" s="24"/>
+    </x:row>
+    <x:row r="116" ht="32" customHeight="1">
+      <x:c r="A116" s="24" t="str">
+        <x:v>PROCEED TO RETRIEVAL DESIGN if both counts are operationally manageable.</x:v>
+      </x:c>
+      <x:c r="B116" s="24"/>
+      <x:c r="C116" s="24"/>
+      <x:c r="D116" s="24"/>
+      <x:c r="E116" s="24"/>
+      <x:c r="F116" s="24"/>
+      <x:c r="G116" s="24"/>
+      <x:c r="H116" s="24"/>
+    </x:row>
+    <x:row r="117" ht="32" customHeight="1">
+      <x:c r="A117" s="24" t="str">
+        <x:v>PARTIAL if only one is manageable. HOLD / REDESIGN if either requires substantive query change.</x:v>
+      </x:c>
+      <x:c r="B117" s="24"/>
+      <x:c r="C117" s="24"/>
+      <x:c r="D117" s="24"/>
+      <x:c r="E117" s="24"/>
+      <x:c r="F117" s="24"/>
+      <x:c r="G117" s="24"/>
+      <x:c r="H117" s="24"/>
+    </x:row>
+    <x:row r="118" ht="32" customHeight="1">
+      <x:c r="A118" s="24" t="str">
+        <x:v>No numeric manageability cutoff supplied. Analyst records capacity rationale and any syntax modifications.</x:v>
+      </x:c>
+      <x:c r="B118" s="24"/>
+      <x:c r="C118" s="24"/>
+      <x:c r="D118" s="24"/>
+      <x:c r="E118" s="24"/>
+      <x:c r="F118" s="24"/>
+      <x:c r="G118" s="24"/>
+      <x:c r="H118" s="24"/>
+    </x:row>
+    <x:row r="119" ht="32" customHeight="1">
+      <x:c r="A119" s="24" t="str">
+        <x:v>Counts only. No GOLD recovery, recall, precision or candidate-family metrics. No searches run during setup.</x:v>
+      </x:c>
+      <x:c r="B119" s="24"/>
+      <x:c r="C119" s="24"/>
+      <x:c r="D119" s="24"/>
+      <x:c r="E119" s="24"/>
+      <x:c r="F119" s="24"/>
+      <x:c r="G119" s="24"/>
+      <x:c r="H119" s="24"/>
+    </x:row>
+    <x:row r="120" ht="32" customHeight="1">
+      <x:c r="A120" s="24" t="str">
+        <x:v>Source: experiments/BC001/EXP-017A/experiment-definition.md</x:v>
+      </x:c>
+      <x:c r="B120" s="24"/>
+      <x:c r="C120" s="24"/>
+      <x:c r="D120" s="24"/>
+      <x:c r="E120" s="24"/>
+      <x:c r="F120" s="24"/>
+      <x:c r="G120" s="24"/>
+      <x:c r="H120" s="24"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1964,6 +2107,17 @@
     <x:mergeCell ref="A97:H97"/>
     <x:mergeCell ref="A98:H98"/>
     <x:mergeCell ref="A99:H99"/>
+    <x:mergeCell ref="A110:H110"/>
+    <x:mergeCell ref="A111:H111"/>
+    <x:mergeCell ref="A112:H112"/>
+    <x:mergeCell ref="A113:H113"/>
+    <x:mergeCell ref="A114:H114"/>
+    <x:mergeCell ref="A115:H115"/>
+    <x:mergeCell ref="A116:H116"/>
+    <x:mergeCell ref="A117:H117"/>
+    <x:mergeCell ref="A118:H118"/>
+    <x:mergeCell ref="A119:H119"/>
+    <x:mergeCell ref="A120:H120"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3011,29 +3165,73 @@
         <x:v>Post-hoc D1 audit; no rerank. Penalty/cap contribution 2/3; title/abstract limits 2/3 (overlapping). EXP-018 semantic extraction proposed only. REJECT unchanged.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="24"/>
-      <x:c r="B20" s="30"/>
-      <x:c r="C20" s="24"/>
-      <x:c r="D20" s="24"/>
-      <x:c r="E20" s="24"/>
-      <x:c r="F20" s="24"/>
-      <x:c r="G20" s="24"/>
-      <x:c r="H20" s="24"/>
-      <x:c r="I20" s="24"/>
-      <x:c r="J20" s="24"/>
-      <x:c r="K20" s="24"/>
-      <x:c r="L20" s="31"/>
-      <x:c r="M20" s="31"/>
-      <x:c r="N20" s="31"/>
-      <x:c r="O20" s="24"/>
-      <x:c r="P20" s="43"/>
-      <x:c r="Q20" s="44"/>
-      <x:c r="R20" s="32"/>
-      <x:c r="S20" s="24"/>
-      <x:c r="T20" s="24"/>
-      <x:c r="U20" s="24"/>
-      <x:c r="V20" s="24"/>
+    <x:row r="20" ht="180" customHeight="1">
+      <x:c r="A20" s="24" t="str">
+        <x:v>EXP-017A</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="C20" s="24" t="str">
+        <x:v>BC001</x:v>
+      </x:c>
+      <x:c r="D20" s="24" t="str">
+        <x:v>0.1-provisional</x:v>
+      </x:c>
+      <x:c r="E20" s="24" t="str">
+        <x:v>EXP-015 recorded Q1/Q2 AND baselines</x:v>
+      </x:c>
+      <x:c r="F20" s="24" t="str">
+        <x:v>Q1P / Q2P unordered 5D</x:v>
+      </x:c>
+      <x:c r="G20" s="24" t="str">
+        <x:v>Determine whether 5D reduces retrieval volume to a practically usable range</x:v>
+      </x:c>
+      <x:c r="H20" s="24" t="str">
+        <x:v>Query Planner / Search Controller</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="str">
+        <x:v>Cross-concept AND</x:v>
+      </x:c>
+      <x:c r="J20" s="24" t="str">
+        <x:v>Unordered 5D</x:v>
+      </x:c>
+      <x:c r="K20" s="24" t="str">
+        <x:v>Only firearm-to-feature operator changes; analyst manual Orbit counts pending</x:v>
+      </x:c>
+      <x:c r="L20" s="31" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="M20" s="31" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N20" s="31" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="O20" s="24" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="P20" s="43" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="Q20" s="44" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="R20" s="32" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="S20" s="24" t="str">
+        <x:v>FAMPAT; TI/AB/CLMS; same vocabulary; no filters or expansion; no benchmark changes</x:v>
+      </x:c>
+      <x:c r="T20" s="24" t="str">
+        <x:v>Pending analyst volume preflight</x:v>
+      </x:c>
+      <x:c r="U20" s="24" t="str">
+        <x:v>AWAITING_ORBIT_PREFLIGHT</x:v>
+      </x:c>
+      <x:c r="V20" s="24" t="str">
+        <x:v>Baselines: Q1 23,935; Q2 493,993 FAMPAT families. Counts only; no searches run at setup. See experiments/BC001/EXP-017A/.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="24"/>
@@ -7403,7 +7601,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f8e6fa386ba449b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9cba65414854bb0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8140,7 +8338,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb71efb718c8c45f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdacafb2b801849d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8557,7 +8755,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6bea4489cbc45dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e861c8d5ee344b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8876,7 +9074,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaf62b19a88a4e10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9042aac8a66c47c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Evaluate and record EXP-018A decision
</commit_message>
<xml_diff>
--- a/Patent_AI_Experiment_Dashboard_Canonical.xlsx
+++ b/Patent_AI_Experiment_Dashboard_Canonical.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb7a666564c424511"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" r:id="R10c2a651947d4766"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Inputs" sheetId="3" r:id="R2beb5e573064478b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Versions" sheetId="4" r:id="R76426214d8914b65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Definitions" sheetId="5" r:id="R9f1ee8d2393b442d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0c6edcd48ed64132"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" r:id="Rd287730fa4e34e63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Inputs" sheetId="3" r:id="Rfd3350348f044237"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Versions" sheetId="4" r:id="Ra5a7bbb3fa684065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Definitions" sheetId="5" r:id="Rf381afedda254aa3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -50,7 +50,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -107,6 +107,16 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -115,7 +125,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="71">
+  <x:cellXfs count="75">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -257,6 +267,10 @@
     <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -640,7 +654,7 @@
       </x:c>
       <x:c r="E5" t="n">
         <x:f>COUNTA('Experiment Log'!A2:A200)</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -648,14 +662,14 @@
         <x:v>Current System</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Retrieval baseline + candidate reranker + validated evidence assist</x:v>
+        <x:v>RUN-012 + EXP-018A + evidence assist</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Promoted experiments</x:v>
       </x:c>
       <x:c r="E6" t="n">
         <x:f>COUNTIF('Experiment Log'!U2:U200,"PROMOTE")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -663,7 +677,7 @@
         <x:v>Current Champion</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>None yet — reranker not promoted</x:v>
+        <x:v>EXP-018A — BC001 TA only</x:v>
       </x:c>
       <x:c r="D7" t="str">
         <x:v>Best Recall@50</x:v>
@@ -678,7 +692,7 @@
         <x:v>Current Experiment</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>EXP-017A</x:v>
+        <x:v>EXP-018A</x:v>
       </x:c>
       <x:c r="D8" t="str">
         <x:v>Best Recall@100</x:v>
@@ -709,7 +723,7 @@
       </x:c>
       <x:c r="E10" s="45" t="n">
         <x:f>MIN('Experiment Log'!P2:P200)</x:f>
-        <x:v>90.5</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2040,6 +2054,179 @@
       <x:c r="F120" s="24"/>
       <x:c r="G120" s="24"/>
       <x:c r="H120" s="24"/>
+    </x:row>
+    <x:row r="123" ht="25" customHeight="1">
+      <x:c r="A123" s="72" t="str">
+        <x:v>EXP-018A — Title/abstract extraction and gating repair</x:v>
+      </x:c>
+      <x:c r="B123" s="72"/>
+      <x:c r="C123" s="72"/>
+      <x:c r="D123" s="72"/>
+      <x:c r="E123" s="72"/>
+      <x:c r="F123" s="72"/>
+      <x:c r="G123" s="72"/>
+      <x:c r="H123" s="72"/>
+    </x:row>
+    <x:row r="124" ht="25" customHeight="1">
+      <x:c r="A124" t="str">
+        <x:v>PROMOTE — recall matches EXP-013; median GOLD rank improves from 90.5 to 55.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="23" customHeight="1">
+      <x:c r="A126" s="74" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B126" s="74" t="str">
+        <x:v>EXP-013</x:v>
+      </x:c>
+      <x:c r="D126" s="74" t="str">
+        <x:v>EXP-016A</x:v>
+      </x:c>
+      <x:c r="E126" s="74" t="str">
+        <x:v>EXP-018A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="23" customHeight="1">
+      <x:c r="A127" t="str">
+        <x:v>Recall@20</x:v>
+      </x:c>
+      <x:c r="B127" s="18" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D127" s="18" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="E127" s="18" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="23" customHeight="1">
+      <x:c r="A128" t="str">
+        <x:v>Recall@50</x:v>
+      </x:c>
+      <x:c r="B128" s="18" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D128" s="18" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="E128" s="18" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="23" customHeight="1">
+      <x:c r="A129" t="str">
+        <x:v>Recall@100</x:v>
+      </x:c>
+      <x:c r="B129" s="18" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="D129" s="18" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E129" s="18" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="23" customHeight="1">
+      <x:c r="A130" t="str">
+        <x:v>Recall@200</x:v>
+      </x:c>
+      <x:c r="B130" s="18" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D130" s="18" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E130" s="18" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="23" customHeight="1">
+      <x:c r="A131" t="str">
+        <x:v>Median GOLD rank</x:v>
+      </x:c>
+      <x:c r="B131" s="45" t="n">
+        <x:v>90.5</x:v>
+      </x:c>
+      <x:c r="D131" s="45" t="n">
+        <x:v>142.5</x:v>
+      </x:c>
+      <x:c r="E131" s="45" t="n">
+        <x:v>55</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="24" customHeight="1">
+      <x:c r="A133" s="36" t="str">
+        <x:v>Recall denominator: GOLD-10. Median: six retrieved families. Top-20 overlap: EXP-013 8/20; EXP-016A 13/20.</x:v>
+      </x:c>
+      <x:c r="B133" s="36"/>
+      <x:c r="C133" s="36"/>
+      <x:c r="D133" s="36"/>
+      <x:c r="E133" s="36"/>
+      <x:c r="F133" s="36"/>
+      <x:c r="G133" s="36"/>
+      <x:c r="H133" s="36"/>
+    </x:row>
+    <x:row r="134" ht="24" customHeight="1">
+      <x:c r="A134" s="36" t="str">
+        <x:v>Affected records: outcomes 7; relationships 61; mechanism 111; storage 63. Sequential counts overlap.</x:v>
+      </x:c>
+      <x:c r="B134" s="36"/>
+      <x:c r="C134" s="36"/>
+      <x:c r="D134" s="36"/>
+      <x:c r="E134" s="36"/>
+      <x:c r="F134" s="36"/>
+      <x:c r="G134" s="36"/>
+      <x:c r="H134" s="36"/>
+    </x:row>
+    <x:row r="135" ht="24" customHeight="1">
+      <x:c r="A135" s="36" t="str">
+        <x:v>All preservation checks passed. Fixed scoring; 66 tests. Ranking committed before private mapping access.</x:v>
+      </x:c>
+      <x:c r="B135" s="36"/>
+      <x:c r="C135" s="36"/>
+      <x:c r="D135" s="36"/>
+      <x:c r="E135" s="36"/>
+      <x:c r="F135" s="36"/>
+      <x:c r="G135" s="36"/>
+      <x:c r="H135" s="36"/>
+    </x:row>
+    <x:row r="136" ht="24" customHeight="1">
+      <x:c r="A136" s="36" t="str">
+        <x:v>Mechanism-general; validated on BC001 only. Diagnosis-informed repair; no cross-domain validation.</x:v>
+      </x:c>
+      <x:c r="B136" s="36"/>
+      <x:c r="C136" s="36"/>
+      <x:c r="D136" s="36"/>
+      <x:c r="E136" s="36"/>
+      <x:c r="F136" s="36"/>
+      <x:c r="G136" s="36"/>
+      <x:c r="H136" s="36"/>
+    </x:row>
+    <x:row r="137" ht="24" customHeight="1">
+      <x:c r="A137" s="36" t="str">
+        <x:v>Individual GOLD ranks remain mixed. Sparse evidence and translated container terminology remain limits.</x:v>
+      </x:c>
+      <x:c r="B137" s="36"/>
+      <x:c r="C137" s="36"/>
+      <x:c r="D137" s="36"/>
+      <x:c r="E137" s="36"/>
+      <x:c r="F137" s="36"/>
+      <x:c r="G137" s="36"/>
+      <x:c r="H137" s="36"/>
+    </x:row>
+    <x:row r="138" ht="24" customHeight="1">
+      <x:c r="A138" s="36" t="str">
+        <x:v>Source: experiments/BC001/EXP-018A/evaluation/evaluation.md</x:v>
+      </x:c>
+      <x:c r="B138" s="36"/>
+      <x:c r="C138" s="36"/>
+      <x:c r="D138" s="36"/>
+      <x:c r="E138" s="36"/>
+      <x:c r="F138" s="36"/>
+      <x:c r="G138" s="36"/>
+      <x:c r="H138" s="36"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2118,6 +2305,14 @@
     <x:mergeCell ref="A118:H118"/>
     <x:mergeCell ref="A119:H119"/>
     <x:mergeCell ref="A120:H120"/>
+    <x:mergeCell ref="A123:H123"/>
+    <x:mergeCell ref="A124:H124"/>
+    <x:mergeCell ref="A133:H133"/>
+    <x:mergeCell ref="A134:H134"/>
+    <x:mergeCell ref="A135:H135"/>
+    <x:mergeCell ref="A136:H136"/>
+    <x:mergeCell ref="A137:H137"/>
+    <x:mergeCell ref="A138:H138"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3233,29 +3428,73 @@
         <x:v>Baselines: Q1 23,935; Q2 493,993 FAMPAT families. Counts only; no searches run at setup. See experiments/BC001/EXP-017A/.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="24"/>
-      <x:c r="B21" s="30"/>
-      <x:c r="C21" s="24"/>
-      <x:c r="D21" s="24"/>
-      <x:c r="E21" s="24"/>
-      <x:c r="F21" s="24"/>
-      <x:c r="G21" s="24"/>
-      <x:c r="H21" s="24"/>
-      <x:c r="I21" s="24"/>
-      <x:c r="J21" s="24"/>
-      <x:c r="K21" s="24"/>
-      <x:c r="L21" s="31"/>
-      <x:c r="M21" s="31"/>
-      <x:c r="N21" s="31"/>
-      <x:c r="O21" s="24"/>
-      <x:c r="P21" s="43"/>
-      <x:c r="Q21" s="44"/>
-      <x:c r="R21" s="32"/>
-      <x:c r="S21" s="24"/>
-      <x:c r="T21" s="24"/>
-      <x:c r="U21" s="24"/>
-      <x:c r="V21" s="24"/>
+    <x:row r="21" ht="100" customHeight="1">
+      <x:c r="A21" s="52" t="str">
+        <x:v>EXP-018A</x:v>
+      </x:c>
+      <x:c r="B21" s="60" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="C21" s="52" t="str">
+        <x:v>BC001</x:v>
+      </x:c>
+      <x:c r="D21" s="52" t="str">
+        <x:v>0.1-provisional</x:v>
+      </x:c>
+      <x:c r="E21" s="52" t="str">
+        <x:v>EXP-013 on RUN-012</x:v>
+      </x:c>
+      <x:c r="F21" s="52" t="str">
+        <x:v>rs_v0.4_extraction_gate_repair_ta</x:v>
+      </x:c>
+      <x:c r="G21" s="52" t="str">
+        <x:v>Repair extraction/gating with fixed scoring and title/abstract evidence</x:v>
+      </x:c>
+      <x:c r="H21" s="52" t="str">
+        <x:v>Relevance Scorer</x:v>
+      </x:c>
+      <x:c r="I21" s="52" t="str">
+        <x:v>rs_v0.3_feature_aware_ta</x:v>
+      </x:c>
+      <x:c r="J21" s="52" t="str">
+        <x:v>rs_v0.4_extraction_gate_repair_ta</x:v>
+      </x:c>
+      <x:c r="K21" s="52" t="str">
+        <x:v>Authentication outcomes; causal linking; functional mechanism; storage/object senses</x:v>
+      </x:c>
+      <x:c r="L21" s="54" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="M21" s="54" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="N21" s="54" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="O21" s="52" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P21" s="61" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="Q21" s="62" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="R21" s="63" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="S21" s="52" t="str">
+        <x:v>R20 2/10; R200 5/10. Individual ranks mixed.</x:v>
+      </x:c>
+      <x:c r="T21" s="52" t="str">
+        <x:v>Recall matches EXP-013; median 90.5 to 55. BC001 only.</x:v>
+      </x:c>
+      <x:c r="U21" s="52" t="str">
+        <x:v>PROMOTE</x:v>
+      </x:c>
+      <x:c r="V21" s="52" t="str">
+        <x:v>Frozen before private mapping. Fixed scoring. 66 tests. TA reranker scope only.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="24"/>
@@ -7601,7 +7840,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9cba65414854bb0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaa11773f8a24f69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8338,7 +8577,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdacafb2b801849d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dbec83153814e6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8563,14 +8802,28 @@
         <x:v>Recall@20 1/10; median GOLD rank 142.5. Rule-based extraction; no promotion.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="24"/>
-      <x:c r="B10" s="24"/>
-      <x:c r="C10" s="24"/>
-      <x:c r="D10" s="24"/>
-      <x:c r="E10" s="24"/>
-      <x:c r="F10" s="24"/>
-      <x:c r="G10" s="24"/>
+    <x:row r="10" ht="65" customHeight="1">
+      <x:c r="A10" s="52" t="str">
+        <x:v>Relevance Scorer</x:v>
+      </x:c>
+      <x:c r="B10" s="52" t="str">
+        <x:v>rs_v0.4_extraction_gate_repair_ta</x:v>
+      </x:c>
+      <x:c r="C10" s="52" t="str">
+        <x:v>PROMOTE; BC001 TA champion</x:v>
+      </x:c>
+      <x:c r="D10" s="52" t="str">
+        <x:v>Extraction/gating repair; fixed scoring</x:v>
+      </x:c>
+      <x:c r="E10" s="52" t="str">
+        <x:v>EXP-018A</x:v>
+      </x:c>
+      <x:c r="F10" s="52" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G10" s="52" t="str">
+        <x:v>Same recall as EXP-013; median 55. BC001 title/abstract only.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="24"/>
@@ -8755,7 +9008,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e861c8d5ee344b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2ffb69331784fdb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9074,7 +9327,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9042aac8a66c47c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc31146219305491f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>